<commit_message>
feature :- chnages in cretae and uplaod mega evnet
</commit_message>
<xml_diff>
--- a/resources/UserDetails_prod.xlsx
+++ b/resources/UserDetails_prod.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Email</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>EldonTrantow@yopmail.com</t>
+  </si>
+  <si>
+    <t>JeramyWest@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1258,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1373,6 +1376,11 @@
         <v>22</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>